<commit_message>
change FrCore dependency to 2.0.1 and correct fsh warnings (#106)
* change dependency and correct fsh warnings

* add downloads page

* fix typo

* update publication-request

* clean aliases page 9935880c92b89ea92b01336401690be9e74ba9d4
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-mesures-observation-glucose.xlsx
+++ b/main/ig/StructureDefinition-mesures-observation-glucose.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-04-25T09:06:15+00:00</t>
+    <t>2024-05-16T08:04:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1331,7 +1331,7 @@
     <t>Observation.subject</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://interopsante.org/fhir/StructureDefinition/FrPatient)
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient)
 </t>
   </si>
   <si>
@@ -1385,7 +1385,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://interopsante.org/fhir/StructureDefinition/FrEncounter)
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-encounter)
 </t>
   </si>
   <si>
@@ -1480,7 +1480,7 @@
     <t>Observation.performer</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(CareTeam|RelatedPerson|http://interopsante.org/fhir/StructureDefinition/FrPractitioner|PractitionerRole|http://interopsante.org/fhir/StructureDefinition/FrOrganization|http://interopsante.org/fhir/StructureDefinition/FrPatient)
+    <t xml:space="preserve">Reference(CareTeam|RelatedPerson|https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-practitioner|PractitionerRole|https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-organization|https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient)
 </t>
   </si>
   <si>
@@ -2614,7 +2614,7 @@
     <col min="8" max="8" width="16.27734375" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="13.26171875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="216.2890625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="223.14453125" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -4802,7 +4802,7 @@
         <v>82</v>
       </c>
       <c r="AN18" t="s" s="2">
-        <v>107</v>
+        <v>82</v>
       </c>
       <c r="AO18" t="s" s="2">
         <v>82</v>

</xml_diff>